<commit_message>
﻿Accept tracker-#1 with review fixes; issue packet tracker-#2 (intake skill)
Review fixes: SETUP.md python.org link corrected + VERIFY tags cleared after cold test; owner wording in dashboard_server.py.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/sample-property/sample-tracker.xlsx
+++ b/fixtures/sample-property/sample-tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sch. E Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Income" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Expenses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sch. E Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Review" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>

</xml_diff>

<commit_message>
Build conversational tracker setup
</commit_message>
<xml_diff>
--- a/fixtures/sample-property/sample-tracker.xlsx
+++ b/fixtures/sample-property/sample-tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Income" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Expenses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Sch. E Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Review" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sch. E Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>

</xml_diff>

<commit_message>
Add propose-only receipt matcher
</commit_message>
<xml_diff>
--- a/fixtures/sample-property/sample-tracker.xlsx
+++ b/fixtures/sample-property/sample-tracker.xlsx
@@ -887,7 +887,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:J13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -912,7 +912,7 @@
     <row r="2" ht="28" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fake source references are relative to this fixture folder. One missing receipt is intentional.</t>
+          <t>Fake source references are relative to this fixture folder. Two empty references test receipt matching.</t>
         </is>
       </c>
     </row>
@@ -1329,14 +1329,50 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr">
-        <is>
-          <t>source-docs/missing-locksmith-receipt.pdf</t>
-        </is>
-      </c>
+      <c r="I12" s="4" t="inlineStr"/>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Intentionally dangling file reference for the demo reconciliation.</t>
+          <t>Intentionally unlinked; its receipt genuinely does not exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="8" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B13" s="4" t="inlineStr">
+        <is>
+          <t>Sample Electric</t>
+        </is>
+      </c>
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Replace porch light fixture</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="inlineStr">
+        <is>
+          <t>L14 — Repairs</t>
+        </is>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>145</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="4" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I13" s="4" t="inlineStr"/>
+      <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Intentionally unlinked; its matching receipt exists in source-docs.</t>
         </is>
       </c>
     </row>
@@ -1345,7 +1381,7 @@
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="A2:J2"/>
   </mergeCells>
-  <conditionalFormatting sqref="J5:J12">
+  <conditionalFormatting sqref="J5:J13">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>ISNUMBER(SEARCH("ACCOUNTANT REVIEW",J5))</formula>
     </cfRule>
@@ -1820,12 +1856,12 @@
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>The tracker points to a file that is not present.</t>
+          <t>No matching receipt is available for the expense row.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Locate the receipt or remove the file reference.</t>
+          <t>Locate the receipt and paste its path into File Reference.</t>
         </is>
       </c>
       <c r="E5" s="4" t="inlineStr">

</xml_diff>

<commit_message>
﻿Accept tracker-#3 + review fix (restore break demo); issue tracker-#4 (packaging)
Review fix: Sample Gardener dangling-reference row restores the fixture's intended reconciler FAIL that tracker-#3 silently removed; check_fixture re-asserts exit 1; SETUP.md updated.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/fixtures/sample-property/sample-tracker.xlsx
+++ b/fixtures/sample-property/sample-tracker.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Income" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenses" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sch. E Summary" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Review" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Income" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Expenses" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sch. E Summary" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Review" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -131,6 +131,7 @@
     <xf numFmtId="165" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -887,7 +888,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J13"/>
+  <dimension ref="A1:J14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1298,16 +1299,16 @@
     </row>
     <row r="12">
       <c r="A12" s="8" t="n">
-        <v>46117</v>
+        <v>46132</v>
       </c>
       <c r="B12" s="4" t="inlineStr">
         <is>
-          <t>Sample Locksmith</t>
+          <t>Sample Gardener</t>
         </is>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Replace rear-entry lock</t>
+          <t>Spring yard cleanup</t>
         </is>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -1316,10 +1317,10 @@
         </is>
       </c>
       <c r="E12" s="5" t="n">
-        <v>95</v>
+        <v>180</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>95</v>
+        <v>180</v>
       </c>
       <c r="G12" s="5" t="n">
         <v>0</v>
@@ -1329,25 +1330,29 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="I12" s="4" t="inlineStr"/>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>source-docs/missing-gardener-invoice.pdf</t>
+        </is>
+      </c>
       <c r="J12" s="4" t="inlineStr">
         <is>
-          <t>Intentionally unlinked; its receipt genuinely does not exist.</t>
+          <t>Intentionally dangling reference — demonstrates the reconciler catching a broken link.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n">
-        <v>46122</v>
+        <v>46117</v>
       </c>
       <c r="B13" s="4" t="inlineStr">
         <is>
-          <t>Sample Electric</t>
+          <t>Sample Locksmith</t>
         </is>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Replace porch light fixture</t>
+          <t>Replace rear-entry lock</t>
         </is>
       </c>
       <c r="D13" s="4" t="inlineStr">
@@ -1356,10 +1361,10 @@
         </is>
       </c>
       <c r="E13" s="5" t="n">
-        <v>145</v>
+        <v>95</v>
       </c>
       <c r="F13" s="5" t="n">
-        <v>145</v>
+        <v>95</v>
       </c>
       <c r="G13" s="5" t="n">
         <v>0</v>
@@ -1371,6 +1376,46 @@
       </c>
       <c r="I13" s="4" t="inlineStr"/>
       <c r="J13" s="4" t="inlineStr">
+        <is>
+          <t>Intentionally unlinked; its receipt genuinely does not exist.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="9" t="n">
+        <v>46122</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sample Electric</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Replace porch light fixture</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>L14 — Repairs</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>145</v>
+      </c>
+      <c r="F14" t="n">
+        <v>145</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>Paid</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr"/>
+      <c r="J14" t="inlineStr">
         <is>
           <t>Intentionally unlinked; its matching receipt exists in source-docs.</t>
         </is>
@@ -1732,34 +1777,34 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="9" t="n"/>
-      <c r="B25" s="10" t="inlineStr">
+      <c r="A25" s="10" t="n"/>
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>20 — Total expenses</t>
         </is>
       </c>
-      <c r="C25" s="11">
+      <c r="C25" s="12">
         <f>SUM(C10:C24)</f>
         <v/>
       </c>
-      <c r="D25" s="10" t="inlineStr">
+      <c r="D25" s="11" t="inlineStr">
         <is>
           <t>Sum of lines 5–19.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="9" t="n"/>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="A26" s="10" t="n"/>
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>21 — Net income</t>
         </is>
       </c>
-      <c r="C26" s="11">
+      <c r="C26" s="12">
         <f>C8+C9-C25</f>
         <v/>
       </c>
-      <c r="D26" s="10" t="inlineStr">
+      <c r="D26" s="11" t="inlineStr">
         <is>
           <t>Line 3 + Line 4 − Line 20.</t>
         </is>

</xml_diff>